<commit_message>
删除变量列: lvgls, BasalRVLS, MedialRVLS, ApicalRVLS
</commit_message>
<xml_diff>
--- a/data/basic_data.xlsx
+++ b/data/basic_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CF5"/>
+  <dimension ref="A1:CB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,125 +714,105 @@
       </c>
       <c r="BH1" t="inlineStr">
         <is>
-          <t>lvgls</t>
+          <t>tr</t>
         </is>
       </c>
       <c r="BI1" t="inlineStr">
         <is>
-          <t>tr</t>
+          <t>pasp</t>
         </is>
       </c>
       <c r="BJ1" t="inlineStr">
         <is>
-          <t>pasp</t>
+          <t>tapse</t>
         </is>
       </c>
       <c r="BK1" t="inlineStr">
         <is>
-          <t>tapse</t>
+          <t>rvs</t>
         </is>
       </c>
       <c r="BL1" t="inlineStr">
         <is>
-          <t>rvs</t>
+          <t>rvfwls</t>
         </is>
       </c>
       <c r="BM1" t="inlineStr">
         <is>
-          <t>rvfwls</t>
+          <t>tapse/pasp</t>
         </is>
       </c>
       <c r="BN1" t="inlineStr">
         <is>
-          <t>tapse/pasp</t>
+          <t>refwls/pasp</t>
         </is>
       </c>
       <c r="BO1" t="inlineStr">
         <is>
-          <t>refwls/pasp</t>
+          <t>rvedv</t>
         </is>
       </c>
       <c r="BP1" t="inlineStr">
         <is>
-          <t>BasalRVLS</t>
+          <t>rvedvi</t>
         </is>
       </c>
       <c r="BQ1" t="inlineStr">
         <is>
-          <t>MedialRVLS</t>
+          <t>rvesv</t>
         </is>
       </c>
       <c r="BR1" t="inlineStr">
         <is>
-          <t>ApicalRVLS</t>
+          <t>rvesvi</t>
         </is>
       </c>
       <c r="BS1" t="inlineStr">
         <is>
-          <t>rvedv</t>
+          <t>rvef</t>
         </is>
       </c>
       <c r="BT1" t="inlineStr">
         <is>
-          <t>rvedvi</t>
+          <t>tyg_tertile</t>
         </is>
       </c>
       <c r="BU1" t="inlineStr">
         <is>
-          <t>rvesv</t>
+          <t>raa</t>
         </is>
       </c>
       <c r="BV1" t="inlineStr">
         <is>
-          <t>rvesvi</t>
+          <t>rav</t>
         </is>
       </c>
       <c r="BW1" t="inlineStr">
         <is>
-          <t>rvef</t>
+          <t>ravi</t>
         </is>
       </c>
       <c r="BX1" t="inlineStr">
         <is>
-          <t>tyg_tertile</t>
+          <t>ra_myopathy</t>
         </is>
       </c>
       <c r="BY1" t="inlineStr">
         <is>
-          <t>raa</t>
+          <t>ra_reservoir</t>
         </is>
       </c>
       <c r="BZ1" t="inlineStr">
         <is>
-          <t>rav</t>
+          <t>ra_reservoir_tertile</t>
         </is>
       </c>
       <c r="CA1" t="inlineStr">
         <is>
-          <t>ravi</t>
+          <t>ra_conduit</t>
         </is>
       </c>
       <c r="CB1" t="inlineStr">
-        <is>
-          <t>ra_myopathy</t>
-        </is>
-      </c>
-      <c r="CC1" t="inlineStr">
-        <is>
-          <t>ra_reservoir</t>
-        </is>
-      </c>
-      <c r="CD1" t="inlineStr">
-        <is>
-          <t>ra_reservoir_tertile</t>
-        </is>
-      </c>
-      <c r="CE1" t="inlineStr">
-        <is>
-          <t>ra_conduit</t>
-        </is>
-      </c>
-      <c r="CF1" t="inlineStr">
         <is>
           <t>ra_booster</t>
         </is>
@@ -1013,78 +993,69 @@
       <c r="BG2" t="n">
         <v>59.5</v>
       </c>
+      <c r="BH2" t="n">
+        <v>1.9</v>
+      </c>
       <c r="BI2" t="n">
-        <v>1.9</v>
+        <v>19</v>
       </c>
       <c r="BJ2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="BK2" t="n">
-        <v>22</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BL2" t="n">
-        <v>8.800000000000001</v>
+        <v>23.4</v>
       </c>
       <c r="BM2" t="n">
-        <v>23.4</v>
+        <v>1.15789473684211</v>
       </c>
       <c r="BN2" t="n">
-        <v>1.15789473684211</v>
+        <v>1.23157894736842</v>
       </c>
       <c r="BO2" t="n">
-        <v>1.23157894736842</v>
+        <v>71</v>
       </c>
       <c r="BP2" t="n">
-        <v>21.4</v>
+        <v>42.0118343195266</v>
       </c>
       <c r="BQ2" t="n">
-        <v>19.1</v>
+        <v>28.471</v>
       </c>
       <c r="BR2" t="n">
-        <v>14.6</v>
+        <v>16.8467455621302</v>
       </c>
       <c r="BS2" t="n">
-        <v>71</v>
-      </c>
-      <c r="BT2" t="n">
-        <v>42.0118343195266</v>
+        <v>59.9</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
       </c>
       <c r="BU2" t="n">
-        <v>28.471</v>
+        <v>16.4</v>
       </c>
       <c r="BV2" t="n">
-        <v>16.8467455621302</v>
+        <v>38.5</v>
       </c>
       <c r="BW2" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
+        <v>22.8</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>0</v>
       </c>
       <c r="BY2" t="n">
-        <v>16.4</v>
+        <v>55.8</v>
       </c>
       <c r="BZ2" t="n">
-        <v>38.5</v>
+        <v>1</v>
       </c>
       <c r="CA2" t="n">
-        <v>22.8</v>
+        <v>36.6333333333333</v>
       </c>
       <c r="CB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CC2" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="CD2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE2" t="n">
-        <v>36.6333333333333</v>
-      </c>
-      <c r="CF2" t="n">
         <v>19.1666666666667</v>
       </c>
     </row>
@@ -1272,78 +1243,69 @@
       <c r="BG3" t="n">
         <v>59.2</v>
       </c>
+      <c r="BH3" t="n">
+        <v>2.4</v>
+      </c>
       <c r="BI3" t="n">
-        <v>2.4</v>
+        <v>28</v>
       </c>
       <c r="BJ3" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="BK3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="BL3" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="BM3" t="n">
-        <v>17</v>
+        <v>0.571428571428571</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.571428571428571</v>
+        <v>0.607142857142857</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.607142857142857</v>
+        <v>170</v>
       </c>
       <c r="BP3" t="n">
-        <v>25.7</v>
+        <v>95.5056179775281</v>
       </c>
       <c r="BQ3" t="n">
-        <v>14.1</v>
+        <v>75.81999999999999</v>
       </c>
       <c r="BR3" t="n">
-        <v>12.6</v>
+        <v>42.5955056179775</v>
       </c>
       <c r="BS3" t="n">
-        <v>170</v>
-      </c>
-      <c r="BT3" t="n">
-        <v>95.5056179775281</v>
+        <v>55.4</v>
+      </c>
+      <c r="BT3" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
       </c>
       <c r="BU3" t="n">
-        <v>75.81999999999999</v>
+        <v>19.8</v>
       </c>
       <c r="BV3" t="n">
-        <v>42.5955056179775</v>
+        <v>60.2</v>
       </c>
       <c r="BW3" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="BX3" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
+        <v>33.8</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>0</v>
       </c>
       <c r="BY3" t="n">
-        <v>19.8</v>
+        <v>54.9</v>
       </c>
       <c r="BZ3" t="n">
-        <v>60.2</v>
+        <v>1</v>
       </c>
       <c r="CA3" t="n">
-        <v>33.8</v>
+        <v>36.0666666666667</v>
       </c>
       <c r="CB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CC3" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="CD3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE3" t="n">
-        <v>36.0666666666667</v>
-      </c>
-      <c r="CF3" t="n">
         <v>18.8333333333333</v>
       </c>
     </row>
@@ -1531,78 +1493,69 @@
       <c r="BG4" t="n">
         <v>59.9</v>
       </c>
+      <c r="BH4" t="n">
+        <v>2.6</v>
+      </c>
       <c r="BI4" t="n">
-        <v>2.6</v>
+        <v>32</v>
       </c>
       <c r="BJ4" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="BK4" t="n">
-        <v>22</v>
+        <v>9.6</v>
       </c>
       <c r="BL4" t="n">
-        <v>9.6</v>
+        <v>22.9</v>
       </c>
       <c r="BM4" t="n">
-        <v>22.9</v>
+        <v>0.6875</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.6875</v>
+        <v>0.715625</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.715625</v>
+        <v>172</v>
       </c>
       <c r="BP4" t="n">
-        <v>21.9</v>
+        <v>110.25641025641</v>
       </c>
       <c r="BQ4" t="n">
-        <v>22.2</v>
+        <v>103.2</v>
       </c>
       <c r="BR4" t="n">
-        <v>14.9</v>
+        <v>66.1538461538462</v>
       </c>
       <c r="BS4" t="n">
-        <v>172</v>
-      </c>
-      <c r="BT4" t="n">
-        <v>110.25641025641</v>
+        <v>40</v>
+      </c>
+      <c r="BT4" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
       </c>
       <c r="BU4" t="n">
-        <v>103.2</v>
+        <v>17.6</v>
       </c>
       <c r="BV4" t="n">
-        <v>66.1538461538462</v>
+        <v>43.1</v>
       </c>
       <c r="BW4" t="n">
-        <v>40</v>
-      </c>
-      <c r="BX4" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
+        <v>27.6</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>0</v>
       </c>
       <c r="BY4" t="n">
-        <v>17.6</v>
+        <v>62.3</v>
       </c>
       <c r="BZ4" t="n">
-        <v>43.1</v>
+        <v>1</v>
       </c>
       <c r="CA4" t="n">
-        <v>27.6</v>
+        <v>46.9</v>
       </c>
       <c r="CB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="CC4" t="n">
-        <v>62.3</v>
-      </c>
-      <c r="CD4" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE4" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="CF4" t="n">
         <v>15.4</v>
       </c>
     </row>
@@ -1788,78 +1741,69 @@
       <c r="BG5" t="n">
         <v>60.5</v>
       </c>
+      <c r="BH5" t="n">
+        <v>3.5</v>
+      </c>
       <c r="BI5" t="n">
-        <v>3.5</v>
+        <v>54</v>
       </c>
       <c r="BJ5" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="BK5" t="n">
-        <v>21</v>
+        <v>9.1</v>
       </c>
       <c r="BL5" t="n">
-        <v>9.1</v>
+        <v>24</v>
       </c>
       <c r="BM5" t="n">
-        <v>24</v>
+        <v>0.388888888888889</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.388888888888889</v>
+        <v>0.444444444444444</v>
       </c>
       <c r="BO5" t="n">
-        <v>0.444444444444444</v>
+        <v>101</v>
       </c>
       <c r="BP5" t="n">
-        <v>30.9</v>
+        <v>47.8672985781991</v>
       </c>
       <c r="BQ5" t="n">
-        <v>32.7</v>
+        <v>52.475</v>
       </c>
       <c r="BR5" t="n">
-        <v>23.6</v>
+        <v>24.8696682464455</v>
       </c>
       <c r="BS5" t="n">
-        <v>101</v>
-      </c>
-      <c r="BT5" t="n">
-        <v>47.8672985781991</v>
+        <v>48</v>
+      </c>
+      <c r="BT5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
       </c>
       <c r="BU5" t="n">
-        <v>52.475</v>
+        <v>17.2</v>
       </c>
       <c r="BV5" t="n">
-        <v>24.8696682464455</v>
+        <v>52.8</v>
       </c>
       <c r="BW5" t="n">
-        <v>48</v>
-      </c>
-      <c r="BX5" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>0</v>
       </c>
       <c r="BY5" t="n">
-        <v>17.2</v>
+        <v>49.8</v>
       </c>
       <c r="BZ5" t="n">
-        <v>52.8</v>
+        <v>1</v>
       </c>
       <c r="CA5" t="n">
-        <v>25</v>
+        <v>19.7</v>
       </c>
       <c r="CB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="CC5" t="n">
-        <v>49.8</v>
-      </c>
-      <c r="CD5" t="n">
-        <v>1</v>
-      </c>
-      <c r="CE5" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="CF5" t="n">
         <v>30.1</v>
       </c>
     </row>

</xml_diff>